<commit_message>
feat: update post-weighing material check template
</commit_message>
<xml_diff>
--- a/backend/templates/post-weighing-material-check-template/post-weighing-material-check-template.xlsx
+++ b/backend/templates/post-weighing-material-check-template/post-weighing-material-check-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phamv\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E26FF74-88A5-4EC0-B5CD-635CDDF71D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3B0163D-B245-452D-95B0-A90EE8FDF639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -380,7 +380,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -389,7 +389,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>